<commit_message>
test(inspect): PRJ-2026-003'u yuksek riske cek (akis testi)
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/projects.xlsx
+++ b/data/projects.xlsx
@@ -398,23 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O7"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="17.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="21.83203125" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" customWidth="1"/>
-    <col min="12" max="12" width="21.83203125" customWidth="1"/>
-    <col min="13" max="13" width="21.83203125" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" customWidth="1"/>
-    <col min="15" max="15" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -571,7 +554,7 @@
         <v>365</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-04-15</v>
+        <v>2027-12-31</v>
       </c>
       <c r="F4" t="str">
         <v>H</v>
@@ -583,22 +566,22 @@
         <v>800000</v>
       </c>
       <c r="I4">
-        <v>780000</v>
+        <v>500000</v>
       </c>
       <c r="J4">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L4">
-        <v>780000</v>
+        <v>500000</v>
       </c>
       <c r="M4">
-        <v>780000</v>
+        <v>750000</v>
       </c>
       <c r="N4">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="O4">
         <v>3</v>
@@ -721,7 +704,7 @@
         <v>H</v>
       </c>
       <c r="H7">
-        <v>7500000</v>
+        <v>75300000</v>
       </c>
       <c r="I7">
         <v>4800000</v>

</xml_diff>